<commit_message>
Sign in with user ID and password, Home split, editors, expense switches
- Sign-in: user ID + password (no list of logins on screen), Super Admin
  resets passwords; passwords stored only hashed. Optional own-data-only
  logins and a Video Editor role.
- Home after sign-in: Diet Charts and Clinic Admin, half the screen each;
  in the app, diet charts need a signed-in login.
- Editors: profiles with a fee per video (default 150, editable), videos
  received from the editor, editor logins see their own videos.
- Expenses: founder card, switches to leave categories or names out of
  totals and profit, per-entry "don't count".
- Purchases: GST on/off per invoice, GST % typed per line, default GST.
- Products: diet plans move up/down and delete.
- Diet charts: line icons in brand colors instead of emoji.
- PDF: info strip with period, prepared by and time.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014wSgWM4oMAShJr56qpgZfC
</commit_message>
<xml_diff>
--- a/admin/ThePrimeFit_Sheets.xlsx
+++ b/admin/ThePrimeFit_Sheets.xlsx
@@ -24,7 +24,8 @@
     <sheet name="Renewals" sheetId="15" state="visible" r:id="rId15"/>
     <sheet name="Doctors" sheetId="16" state="visible" r:id="rId16"/>
     <sheet name="Content" sheetId="17" state="visible" r:id="rId17"/>
-    <sheet name="Activity Log" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet name="Editors" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet name="Activity Log" sheetId="19" state="visible" r:id="rId19"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -193,6 +194,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -489,7 +493,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A8:A21"/>
+  <dimension ref="A8:A29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="120" customWidth="1" min="1" max="1"/>
@@ -567,7 +571,7 @@
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>The app saves all data here. Each save rewrites the 17 sheets (Dashboard … Activity Log, including Doctors and Content), so edit data in the app, not in the sheets.</t>
+          <t>The app saves all data here. Each save rewrites the 18 sheets (Dashboard … Activity Log, including Doctors, Editors and Content), so edit data in the app, not in the sheets.</t>
         </is>
       </c>
     </row>
@@ -585,6 +589,14 @@
         </is>
       </c>
     </row>
+    <row r="22"/>
+    <row r="23"/>
+    <row r="24"/>
+    <row r="25"/>
+    <row r="26"/>
+    <row r="27"/>
+    <row r="28"/>
+    <row r="29"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -1481,7 +1493,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F1"/>
+  <dimension ref="A1:G1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1490,6 +1502,7 @@
     <col width="12" customWidth="1" min="4" max="4"/>
     <col width="17" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1521,6 +1534,11 @@
       <c r="F1" s="4" t="inlineStr">
         <is>
           <t>Note</t>
+        </is>
+      </c>
+      <c r="G1" s="4" t="inlineStr">
+        <is>
+          <t>Counted</t>
         </is>
       </c>
     </row>
@@ -1676,7 +1694,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J1"/>
+  <dimension ref="A1:K1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1686,9 +1704,10 @@
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
     <col width="12" customWidth="1" min="7" max="7"/>
-    <col width="15" customWidth="1" min="8" max="8"/>
-    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="13" customWidth="1" min="9" max="9"/>
     <col width="12" customWidth="1" min="10" max="10"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1719,25 +1738,30 @@
       </c>
       <c r="F1" s="4" t="inlineStr">
         <is>
+          <t>Received</t>
+        </is>
+      </c>
+      <c r="G1" s="4" t="inlineStr">
+        <is>
           <t>Scheduled</t>
         </is>
       </c>
-      <c r="G1" s="4" t="inlineStr">
+      <c r="H1" s="4" t="inlineStr">
         <is>
           <t>Posted</t>
         </is>
       </c>
-      <c r="H1" s="4" t="inlineStr">
-        <is>
-          <t>Editing Cost</t>
-        </is>
-      </c>
       <c r="I1" s="4" t="inlineStr">
         <is>
+          <t>Editor Fee</t>
+        </is>
+      </c>
+      <c r="J1" s="4" t="inlineStr">
+        <is>
           <t>Link</t>
         </is>
       </c>
-      <c r="J1" s="4" t="inlineStr">
+      <c r="K1" s="4" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
@@ -1749,6 +1773,67 @@
 </file>
 
 <file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="00015B53"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B1" s="4" t="inlineStr">
+        <is>
+          <t>Mobile</t>
+        </is>
+      </c>
+      <c r="C1" s="4" t="inlineStr">
+        <is>
+          <t>Fee per Video</t>
+        </is>
+      </c>
+      <c r="D1" s="4" t="inlineStr">
+        <is>
+          <t>Videos Received</t>
+        </is>
+      </c>
+      <c r="E1" s="4" t="inlineStr">
+        <is>
+          <t>Videos Posted</t>
+        </is>
+      </c>
+      <c r="F1" s="4" t="inlineStr">
+        <is>
+          <t>Total Fees</t>
+        </is>
+      </c>
+      <c r="G1" s="4" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="00015B53"/>
@@ -2233,7 +2318,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>2026-10-01T16:36:33.841Z</t>
+          <t>2026-10-01T17:12:29.724Z</t>
         </is>
       </c>
       <c r="C34" t="inlineStr"/>

</xml_diff>

<commit_message>
Admin: product types, clinics, Customize, WhatsApp card, lead summary, themes
- No starter injections, protein, supplies or diet plans (unused ones removed
  from older data); clinics create their own product types
- Multiple OPD clinics on appointments, filters, dashboard and OPD slip
- Customize on summary screens to show or hide any card or box
- WhatsApp today card, lead daily summary and follow-up reminders
- Social counts read the public YouTube/Instagram pages without keys
- Five themes with light/dark mode, plate cards, menu search and quick actions

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014wSgWM4oMAShJr56qpgZfC
</commit_message>
<xml_diff>
--- a/admin/ThePrimeFit_Sheets.xlsx
+++ b/admin/ThePrimeFit_Sheets.xlsx
@@ -15,18 +15,19 @@
     <sheet name="Injection Sales" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="Protein Sales" sheetId="7" state="visible" r:id="rId7"/>
     <sheet name="Diet Support" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="Service Sales" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="Purchases" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="Inventory" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="Team" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="Incentives" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet name="Salary" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet name="Expenses" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet name="Renewals" sheetId="16" state="visible" r:id="rId16"/>
-    <sheet name="Doctors" sheetId="17" state="visible" r:id="rId17"/>
-    <sheet name="Content" sheetId="18" state="visible" r:id="rId18"/>
-    <sheet name="Editors" sheetId="19" state="visible" r:id="rId19"/>
-    <sheet name="Activity Log" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet name="Other Sales" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Service Sales" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="Purchases" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="Inventory" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="Team" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="Incentives" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet name="Salary" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet name="Expenses" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet name="Renewals" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet name="Doctors" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet name="Content" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet name="Editors" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet name="Activity Log" sheetId="21" state="visible" r:id="rId21"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -580,7 +581,7 @@
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>The app saves all data here. Each save rewrites the 19 sheets (Dashboard … Activity Log, including Service Sales, Doctors, Editors and Content), so edit data in the app, not in the sheets.</t>
+          <t>The app saves all data here. Each save rewrites the 20 sheets (Dashboard … Activity Log, including Service Sales, Other Sales, Doctors, Editors and Content), so edit data in the app, not in the sheets.</t>
         </is>
       </c>
     </row>
@@ -605,6 +606,96 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:L1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="19" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="18" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="10" max="10"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="5" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="B1" s="5" t="inlineStr">
+        <is>
+          <t>Patient</t>
+        </is>
+      </c>
+      <c r="C1" s="5" t="inlineStr">
+        <is>
+          <t>Mobile</t>
+        </is>
+      </c>
+      <c r="D1" s="5" t="inlineStr">
+        <is>
+          <t>New/Renewal</t>
+        </is>
+      </c>
+      <c r="E1" s="5" t="inlineStr">
+        <is>
+          <t>Service / Package</t>
+        </is>
+      </c>
+      <c r="F1" s="5" t="inlineStr">
+        <is>
+          <t>Qty</t>
+        </is>
+      </c>
+      <c r="G1" s="5" t="inlineStr">
+        <is>
+          <t>Amount</t>
+        </is>
+      </c>
+      <c r="H1" s="5" t="inlineStr">
+        <is>
+          <t>Reference</t>
+        </is>
+      </c>
+      <c r="I1" s="5" t="inlineStr">
+        <is>
+          <t>Shared Reference</t>
+        </is>
+      </c>
+      <c r="J1" s="5" t="inlineStr">
+        <is>
+          <t>Split</t>
+        </is>
+      </c>
+      <c r="K1" s="5" t="inlineStr">
+        <is>
+          <t>Incentive</t>
+        </is>
+      </c>
+      <c r="L1" s="5" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -688,13 +779,13 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K20"/>
+  <dimension ref="A1:K5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="23" customWidth="1" min="1" max="1"/>
@@ -770,16 +861,18 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Injection</t>
+          <t>GLP-1 Success Support</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Mounjaro 2.5mg</t>
-        </is>
-      </c>
-      <c r="C2" t="n">
-        <v>0</v>
+          <t>GLP-1 Success Support · 1 Week</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Unlimited</t>
+        </is>
       </c>
       <c r="D2" t="n">
         <v>0</v>
@@ -793,31 +886,34 @@
       <c r="G2" t="n">
         <v>0</v>
       </c>
-      <c r="H2" t="n">
-        <v>0</v>
-      </c>
-      <c r="I2" t="n">
-        <v>2</v>
-      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Unlimited</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr"/>
       <c r="J2" t="inlineStr">
         <is>
-          <t>LOW</t>
-        </is>
-      </c>
+          <t>Service</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Injection</t>
+          <t>GLP-1 Success Support</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Mounjaro 5mg</t>
-        </is>
-      </c>
-      <c r="C3" t="n">
-        <v>0</v>
+          <t>GLP-1 Success Support · 1 Month</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Unlimited</t>
+        </is>
       </c>
       <c r="D3" t="n">
         <v>0</v>
@@ -831,31 +927,34 @@
       <c r="G3" t="n">
         <v>0</v>
       </c>
-      <c r="H3" t="n">
-        <v>0</v>
-      </c>
-      <c r="I3" t="n">
-        <v>2</v>
-      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Unlimited</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr"/>
       <c r="J3" t="inlineStr">
         <is>
-          <t>LOW</t>
-        </is>
-      </c>
+          <t>Service</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Injection</t>
+          <t>GLP-1 Success Support</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Mounjaro 10mg</t>
-        </is>
-      </c>
-      <c r="C4" t="n">
-        <v>0</v>
+          <t>GLP-1 Success Support · 2 Months</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Unlimited</t>
+        </is>
       </c>
       <c r="D4" t="n">
         <v>0</v>
@@ -869,36 +968,34 @@
       <c r="G4" t="n">
         <v>0</v>
       </c>
-      <c r="H4" t="n">
-        <v>0</v>
-      </c>
-      <c r="I4" t="n">
-        <v>2</v>
-      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Unlimited</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr"/>
       <c r="J4" t="inlineStr">
         <is>
-          <t>LOW</t>
-        </is>
-      </c>
-      <c r="K4" t="inlineStr">
-        <is>
-          <t>ORDER REQUIRED</t>
-        </is>
-      </c>
+          <t>Service</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Injection</t>
+          <t>GLP-1 Success Support</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Mounjaro 15mg</t>
-        </is>
-      </c>
-      <c r="C5" t="n">
-        <v>0</v>
+          <t>GLP-1 Success Support · 3 Months</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Unlimited</t>
+        </is>
       </c>
       <c r="D5" t="n">
         <v>0</v>
@@ -912,608 +1009,25 @@
       <c r="G5" t="n">
         <v>0</v>
       </c>
-      <c r="H5" t="n">
-        <v>0</v>
-      </c>
-      <c r="I5" t="n">
-        <v>2</v>
-      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Unlimited</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr"/>
       <c r="J5" t="inlineStr">
         <is>
-          <t>LOW</t>
-        </is>
-      </c>
-      <c r="K5" t="inlineStr">
-        <is>
-          <t>ORDER REQUIRED</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Injection</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>Wegovy 0.25mg</t>
-        </is>
-      </c>
-      <c r="C6" t="n">
-        <v>0</v>
-      </c>
-      <c r="D6" t="n">
-        <v>0</v>
-      </c>
-      <c r="E6" t="n">
-        <v>0</v>
-      </c>
-      <c r="F6" t="n">
-        <v>0</v>
-      </c>
-      <c r="G6" t="n">
-        <v>0</v>
-      </c>
-      <c r="H6" t="n">
-        <v>0</v>
-      </c>
-      <c r="I6" t="n">
-        <v>2</v>
-      </c>
-      <c r="J6" t="inlineStr">
-        <is>
-          <t>LOW</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>Injection</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>Wegovy 1mg</t>
-        </is>
-      </c>
-      <c r="C7" t="n">
-        <v>0</v>
-      </c>
-      <c r="D7" t="n">
-        <v>0</v>
-      </c>
-      <c r="E7" t="n">
-        <v>0</v>
-      </c>
-      <c r="F7" t="n">
-        <v>0</v>
-      </c>
-      <c r="G7" t="n">
-        <v>0</v>
-      </c>
-      <c r="H7" t="n">
-        <v>0</v>
-      </c>
-      <c r="I7" t="n">
-        <v>2</v>
-      </c>
-      <c r="J7" t="inlineStr">
-        <is>
-          <t>LOW</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>Injection</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>Wegovy 2.4mg</t>
-        </is>
-      </c>
-      <c r="C8" t="n">
-        <v>0</v>
-      </c>
-      <c r="D8" t="n">
-        <v>0</v>
-      </c>
-      <c r="E8" t="n">
-        <v>0</v>
-      </c>
-      <c r="F8" t="n">
-        <v>0</v>
-      </c>
-      <c r="G8" t="n">
-        <v>0</v>
-      </c>
-      <c r="H8" t="n">
-        <v>0</v>
-      </c>
-      <c r="I8" t="n">
-        <v>2</v>
-      </c>
-      <c r="J8" t="inlineStr">
-        <is>
-          <t>LOW</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>Injection</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>Ozempic 0.25mg</t>
-        </is>
-      </c>
-      <c r="C9" t="n">
-        <v>0</v>
-      </c>
-      <c r="D9" t="n">
-        <v>0</v>
-      </c>
-      <c r="E9" t="n">
-        <v>0</v>
-      </c>
-      <c r="F9" t="n">
-        <v>0</v>
-      </c>
-      <c r="G9" t="n">
-        <v>0</v>
-      </c>
-      <c r="H9" t="n">
-        <v>0</v>
-      </c>
-      <c r="I9" t="n">
-        <v>2</v>
-      </c>
-      <c r="J9" t="inlineStr">
-        <is>
-          <t>LOW</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>Injection</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>Ozempic 1mg</t>
-        </is>
-      </c>
-      <c r="C10" t="n">
-        <v>0</v>
-      </c>
-      <c r="D10" t="n">
-        <v>0</v>
-      </c>
-      <c r="E10" t="n">
-        <v>0</v>
-      </c>
-      <c r="F10" t="n">
-        <v>0</v>
-      </c>
-      <c r="G10" t="n">
-        <v>0</v>
-      </c>
-      <c r="H10" t="n">
-        <v>0</v>
-      </c>
-      <c r="I10" t="n">
-        <v>2</v>
-      </c>
-      <c r="J10" t="inlineStr">
-        <is>
-          <t>LOW</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>Protein</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>Protein Sachets</t>
-        </is>
-      </c>
-      <c r="C11" t="n">
-        <v>0</v>
-      </c>
-      <c r="D11" t="n">
-        <v>0</v>
-      </c>
-      <c r="E11" t="n">
-        <v>0</v>
-      </c>
-      <c r="F11" t="n">
-        <v>0</v>
-      </c>
-      <c r="G11" t="n">
-        <v>0</v>
-      </c>
-      <c r="H11" t="n">
-        <v>0</v>
-      </c>
-      <c r="I11" t="n">
-        <v>20</v>
-      </c>
-      <c r="J11" t="inlineStr">
-        <is>
-          <t>LOW</t>
-        </is>
-      </c>
-      <c r="K11" t="inlineStr">
-        <is>
-          <t>ORDER REQUIRED</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>GLP-1 Success Support</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>GLP-1 Success Support · 1 Week</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>Unlimited</t>
-        </is>
-      </c>
-      <c r="D12" t="n">
-        <v>0</v>
-      </c>
-      <c r="E12" t="n">
-        <v>0</v>
-      </c>
-      <c r="F12" t="n">
-        <v>0</v>
-      </c>
-      <c r="G12" t="n">
-        <v>0</v>
-      </c>
-      <c r="H12" t="inlineStr">
-        <is>
-          <t>Unlimited</t>
-        </is>
-      </c>
-      <c r="J12" t="inlineStr">
-        <is>
           <t>Service</t>
         </is>
       </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>GLP-1 Success Support</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>GLP-1 Success Support · 1 Month</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>Unlimited</t>
-        </is>
-      </c>
-      <c r="D13" t="n">
-        <v>0</v>
-      </c>
-      <c r="E13" t="n">
-        <v>0</v>
-      </c>
-      <c r="F13" t="n">
-        <v>0</v>
-      </c>
-      <c r="G13" t="n">
-        <v>0</v>
-      </c>
-      <c r="H13" t="inlineStr">
-        <is>
-          <t>Unlimited</t>
-        </is>
-      </c>
-      <c r="J13" t="inlineStr">
-        <is>
-          <t>Service</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>GLP-1 Success Support</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>GLP-1 Success Support · 2 Months</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>Unlimited</t>
-        </is>
-      </c>
-      <c r="D14" t="n">
-        <v>0</v>
-      </c>
-      <c r="E14" t="n">
-        <v>0</v>
-      </c>
-      <c r="F14" t="n">
-        <v>0</v>
-      </c>
-      <c r="G14" t="n">
-        <v>0</v>
-      </c>
-      <c r="H14" t="inlineStr">
-        <is>
-          <t>Unlimited</t>
-        </is>
-      </c>
-      <c r="J14" t="inlineStr">
-        <is>
-          <t>Service</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>GLP-1 Success Support</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>GLP-1 Success Support · 3 Months</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>Unlimited</t>
-        </is>
-      </c>
-      <c r="D15" t="n">
-        <v>0</v>
-      </c>
-      <c r="E15" t="n">
-        <v>0</v>
-      </c>
-      <c r="F15" t="n">
-        <v>0</v>
-      </c>
-      <c r="G15" t="n">
-        <v>0</v>
-      </c>
-      <c r="H15" t="inlineStr">
-        <is>
-          <t>Unlimited</t>
-        </is>
-      </c>
-      <c r="J15" t="inlineStr">
-        <is>
-          <t>Service</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>Needles</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>Needles</t>
-        </is>
-      </c>
-      <c r="C16" t="n">
-        <v>0</v>
-      </c>
-      <c r="D16" t="n">
-        <v>0</v>
-      </c>
-      <c r="E16" t="n">
-        <v>0</v>
-      </c>
-      <c r="F16" t="n">
-        <v>0</v>
-      </c>
-      <c r="G16" t="n">
-        <v>0</v>
-      </c>
-      <c r="H16" t="n">
-        <v>0</v>
-      </c>
-      <c r="I16" t="n">
-        <v>20</v>
-      </c>
-      <c r="J16" t="inlineStr">
-        <is>
-          <t>LOW</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>Alcohol Swabs</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>Alcohol Swabs</t>
-        </is>
-      </c>
-      <c r="C17" t="n">
-        <v>0</v>
-      </c>
-      <c r="D17" t="n">
-        <v>0</v>
-      </c>
-      <c r="E17" t="n">
-        <v>0</v>
-      </c>
-      <c r="F17" t="n">
-        <v>0</v>
-      </c>
-      <c r="G17" t="n">
-        <v>0</v>
-      </c>
-      <c r="H17" t="n">
-        <v>0</v>
-      </c>
-      <c r="I17" t="n">
-        <v>20</v>
-      </c>
-      <c r="J17" t="inlineStr">
-        <is>
-          <t>LOW</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>Insulin Syringes</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>Insulin Syringes</t>
-        </is>
-      </c>
-      <c r="C18" t="n">
-        <v>0</v>
-      </c>
-      <c r="D18" t="n">
-        <v>0</v>
-      </c>
-      <c r="E18" t="n">
-        <v>0</v>
-      </c>
-      <c r="F18" t="n">
-        <v>0</v>
-      </c>
-      <c r="G18" t="n">
-        <v>0</v>
-      </c>
-      <c r="H18" t="n">
-        <v>0</v>
-      </c>
-      <c r="I18" t="n">
-        <v>20</v>
-      </c>
-      <c r="J18" t="inlineStr">
-        <is>
-          <t>LOW</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>Ice Gel Packs</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>Ice Gel Packs</t>
-        </is>
-      </c>
-      <c r="C19" t="n">
-        <v>0</v>
-      </c>
-      <c r="D19" t="n">
-        <v>0</v>
-      </c>
-      <c r="E19" t="n">
-        <v>0</v>
-      </c>
-      <c r="F19" t="n">
-        <v>0</v>
-      </c>
-      <c r="G19" t="n">
-        <v>0</v>
-      </c>
-      <c r="H19" t="n">
-        <v>0</v>
-      </c>
-      <c r="I19" t="n">
-        <v>20</v>
-      </c>
-      <c r="J19" t="inlineStr">
-        <is>
-          <t>LOW</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>Travel Bags</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>Travel Bags</t>
-        </is>
-      </c>
-      <c r="C20" t="n">
-        <v>0</v>
-      </c>
-      <c r="D20" t="n">
-        <v>0</v>
-      </c>
-      <c r="E20" t="n">
-        <v>0</v>
-      </c>
-      <c r="F20" t="n">
-        <v>0</v>
-      </c>
-      <c r="G20" t="n">
-        <v>0</v>
-      </c>
-      <c r="H20" t="n">
-        <v>0</v>
-      </c>
-      <c r="I20" t="n">
-        <v>20</v>
-      </c>
-      <c r="J20" t="inlineStr">
-        <is>
-          <t>LOW</t>
-        </is>
-      </c>
+      <c r="K5" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1591,7 +1105,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1651,7 +1165,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1711,7 +1225,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1771,7 +1285,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1837,7 +1351,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1909,7 +1423,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1993,7 +1507,438 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C34"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="5" t="inlineStr">
+        <is>
+          <t>Metric</t>
+        </is>
+      </c>
+      <c r="B1" s="5" t="inlineStr">
+        <is>
+          <t>This month</t>
+        </is>
+      </c>
+      <c r="C1" s="5" t="inlineStr">
+        <is>
+          <t>All time</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Total Orders</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>0</v>
+      </c>
+      <c r="C2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Total Revenue</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Total Expenses</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>0</v>
+      </c>
+      <c r="C4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Net Profit</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Injection Sales</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Protein Sales</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Diet Support Sales</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>0</v>
+      </c>
+      <c r="C8" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Consultation Fees</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>0</v>
+      </c>
+      <c r="C9" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Appointments</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>0</v>
+      </c>
+      <c r="C10" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Clinic Visits</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>0</v>
+      </c>
+      <c r="C11" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Online Consultations</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>0</v>
+      </c>
+      <c r="C12" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>New Leads</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>0</v>
+      </c>
+      <c r="C13" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Leads Converted</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>0</v>
+      </c>
+      <c r="C14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Open Leads</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>0</v>
+      </c>
+      <c r="C15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Order Required</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr"/>
+      <c r="C16" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Total Patients</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>0</v>
+      </c>
+      <c r="C17" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>New Patients</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>0</v>
+      </c>
+      <c r="C18" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Renewal Patients</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>0</v>
+      </c>
+      <c r="C19" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Active Patients</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>0</v>
+      </c>
+      <c r="C20" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Team Members</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>0</v>
+      </c>
+      <c r="C21" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Total Incentives</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>0</v>
+      </c>
+      <c r="C22" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Monthly Salary</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>0</v>
+      </c>
+      <c r="C23" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Top Performer</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr"/>
+      <c r="C24" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Injection Stock</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>0</v>
+      </c>
+      <c r="C25" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Protein Stock</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>0</v>
+      </c>
+      <c r="C26" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Needles Stock</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>0</v>
+      </c>
+      <c r="C27" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Swabs Stock</t>
+        </is>
+      </c>
+      <c r="B28" t="n">
+        <v>0</v>
+      </c>
+      <c r="C28" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Syringe Stock</t>
+        </is>
+      </c>
+      <c r="B29" t="n">
+        <v>0</v>
+      </c>
+      <c r="C29" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Low Stock Alerts</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr"/>
+      <c r="C30" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Videos Edited</t>
+        </is>
+      </c>
+      <c r="B31" t="n">
+        <v>0</v>
+      </c>
+      <c r="C31" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Videos Posted</t>
+        </is>
+      </c>
+      <c r="B32" t="n">
+        <v>0</v>
+      </c>
+      <c r="C32" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Videos Remaining</t>
+        </is>
+      </c>
+      <c r="B33" t="n">
+        <v>0</v>
+      </c>
+      <c r="C33" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Updated</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>2026-10-01T18:34:37.012Z</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2053,448 +1998,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:C34"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="22" customWidth="1" min="1" max="1"/>
-    <col width="50" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="5" t="inlineStr">
-        <is>
-          <t>Metric</t>
-        </is>
-      </c>
-      <c r="B1" s="5" t="inlineStr">
-        <is>
-          <t>This month</t>
-        </is>
-      </c>
-      <c r="C1" s="5" t="inlineStr">
-        <is>
-          <t>All time</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Total Orders</t>
-        </is>
-      </c>
-      <c r="B2" t="n">
-        <v>0</v>
-      </c>
-      <c r="C2" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Total Revenue</t>
-        </is>
-      </c>
-      <c r="B3" t="n">
-        <v>0</v>
-      </c>
-      <c r="C3" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Total Expenses</t>
-        </is>
-      </c>
-      <c r="B4" t="n">
-        <v>0</v>
-      </c>
-      <c r="C4" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Net Profit</t>
-        </is>
-      </c>
-      <c r="B5" t="n">
-        <v>0</v>
-      </c>
-      <c r="C5" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Injection Sales</t>
-        </is>
-      </c>
-      <c r="B6" t="n">
-        <v>0</v>
-      </c>
-      <c r="C6" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>Protein Sales</t>
-        </is>
-      </c>
-      <c r="B7" t="n">
-        <v>0</v>
-      </c>
-      <c r="C7" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>Diet Support Sales</t>
-        </is>
-      </c>
-      <c r="B8" t="n">
-        <v>0</v>
-      </c>
-      <c r="C8" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>Consultation Fees</t>
-        </is>
-      </c>
-      <c r="B9" t="n">
-        <v>0</v>
-      </c>
-      <c r="C9" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>Appointments</t>
-        </is>
-      </c>
-      <c r="B10" t="n">
-        <v>0</v>
-      </c>
-      <c r="C10" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>Clinic Visits</t>
-        </is>
-      </c>
-      <c r="B11" t="n">
-        <v>0</v>
-      </c>
-      <c r="C11" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>Online Consultations</t>
-        </is>
-      </c>
-      <c r="B12" t="n">
-        <v>0</v>
-      </c>
-      <c r="C12" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>New Leads</t>
-        </is>
-      </c>
-      <c r="B13" t="n">
-        <v>0</v>
-      </c>
-      <c r="C13" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>Leads Converted</t>
-        </is>
-      </c>
-      <c r="B14" t="n">
-        <v>0</v>
-      </c>
-      <c r="C14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>Open Leads</t>
-        </is>
-      </c>
-      <c r="B15" t="n">
-        <v>0</v>
-      </c>
-      <c r="C15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>Order Required</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>Mounjaro 10mg (0), Mounjaro 15mg (0), Protein Sachets (0)</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>Total Patients</t>
-        </is>
-      </c>
-      <c r="B17" t="n">
-        <v>0</v>
-      </c>
-      <c r="C17" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>New Patients</t>
-        </is>
-      </c>
-      <c r="B18" t="n">
-        <v>0</v>
-      </c>
-      <c r="C18" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>Renewal Patients</t>
-        </is>
-      </c>
-      <c r="B19" t="n">
-        <v>0</v>
-      </c>
-      <c r="C19" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>Active Patients</t>
-        </is>
-      </c>
-      <c r="B20" t="n">
-        <v>0</v>
-      </c>
-      <c r="C20" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>Team Members</t>
-        </is>
-      </c>
-      <c r="B21" t="n">
-        <v>0</v>
-      </c>
-      <c r="C21" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>Total Incentives</t>
-        </is>
-      </c>
-      <c r="B22" t="n">
-        <v>0</v>
-      </c>
-      <c r="C22" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>Monthly Salary</t>
-        </is>
-      </c>
-      <c r="B23" t="n">
-        <v>0</v>
-      </c>
-      <c r="C23" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>Top Performer</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>Injection Stock</t>
-        </is>
-      </c>
-      <c r="B25" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>Protein Stock</t>
-        </is>
-      </c>
-      <c r="B26" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>Needles Stock</t>
-        </is>
-      </c>
-      <c r="B27" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>Swabs Stock</t>
-        </is>
-      </c>
-      <c r="B28" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>Syringe Stock</t>
-        </is>
-      </c>
-      <c r="B29" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>Low Stock Alerts</t>
-        </is>
-      </c>
-      <c r="B30" t="inlineStr">
-        <is>
-          <t>Mounjaro 2.5mg (0), Mounjaro 5mg (0), Mounjaro 10mg (0), Mounjaro 15mg (0), Wegovy 0.25mg (0), Wegovy 1mg (0), Wegovy 2.4mg (0), Ozempic 0.25mg (0), Ozempic 1mg (0), Protein Sachets (0), Needles (0), Alcohol Swabs (0), Insulin Syringes (0), Ice Gel Packs (0), Travel Bags (0)</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t>Videos Edited</t>
-        </is>
-      </c>
-      <c r="B31" t="n">
-        <v>0</v>
-      </c>
-      <c r="C31" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>Videos Posted</t>
-        </is>
-      </c>
-      <c r="B32" t="n">
-        <v>0</v>
-      </c>
-      <c r="C32" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="inlineStr">
-        <is>
-          <t>Videos Remaining</t>
-        </is>
-      </c>
-      <c r="B33" t="n">
-        <v>0</v>
-      </c>
-      <c r="C33" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" t="inlineStr">
-        <is>
-          <t>Updated</t>
-        </is>
-      </c>
-      <c r="B34" t="inlineStr">
-        <is>
-          <t>2026-10-01T17:49:06.989Z</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2542,7 +2046,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M1"/>
+  <dimension ref="A1:N1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2554,10 +2058,11 @@
     <col width="12" customWidth="1" min="7" max="7"/>
     <col width="12" customWidth="1" min="8" max="8"/>
     <col width="12" customWidth="1" min="9" max="9"/>
-    <col width="16" customWidth="1" min="10" max="10"/>
-    <col width="12" customWidth="1" min="11" max="11"/>
-    <col width="13" customWidth="1" min="12" max="12"/>
-    <col width="12" customWidth="1" min="13" max="13"/>
+    <col width="12" customWidth="1" min="10" max="10"/>
+    <col width="16" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="13" customWidth="1" min="13" max="13"/>
+    <col width="12" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2588,40 +2093,45 @@
       </c>
       <c r="F1" s="5" t="inlineStr">
         <is>
+          <t>Clinic</t>
+        </is>
+      </c>
+      <c r="G1" s="5" t="inlineStr">
+        <is>
           <t>Doctor</t>
         </is>
       </c>
-      <c r="G1" s="5" t="inlineStr">
+      <c r="H1" s="5" t="inlineStr">
         <is>
           <t>Service</t>
         </is>
       </c>
-      <c r="H1" s="5" t="inlineStr">
+      <c r="I1" s="5" t="inlineStr">
         <is>
           <t>Fee</t>
         </is>
       </c>
-      <c r="I1" s="5" t="inlineStr">
+      <c r="J1" s="5" t="inlineStr">
         <is>
           <t>Payment</t>
         </is>
       </c>
-      <c r="J1" s="5" t="inlineStr">
+      <c r="K1" s="5" t="inlineStr">
         <is>
           <t>Payment Method</t>
         </is>
       </c>
-      <c r="K1" s="5" t="inlineStr">
+      <c r="L1" s="5" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="L1" s="5" t="inlineStr">
+      <c r="M1" s="5" t="inlineStr">
         <is>
           <t>Online Link</t>
         </is>
       </c>
-      <c r="M1" s="5" t="inlineStr">
+      <c r="N1" s="5" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
@@ -3100,21 +2610,22 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L1"/>
+  <dimension ref="A1:M1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="13" customWidth="1" min="4" max="4"/>
-    <col width="19" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
     <col width="12" customWidth="1" min="7" max="7"/>
     <col width="12" customWidth="1" min="8" max="8"/>
-    <col width="18" customWidth="1" min="9" max="9"/>
-    <col width="12" customWidth="1" min="10" max="10"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="18" customWidth="1" min="10" max="10"/>
     <col width="12" customWidth="1" min="11" max="11"/>
     <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="12" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3125,55 +2636,60 @@
       </c>
       <c r="B1" s="5" t="inlineStr">
         <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="C1" s="5" t="inlineStr">
+        <is>
           <t>Patient</t>
         </is>
       </c>
-      <c r="C1" s="5" t="inlineStr">
+      <c r="D1" s="5" t="inlineStr">
         <is>
           <t>Mobile</t>
         </is>
       </c>
-      <c r="D1" s="5" t="inlineStr">
+      <c r="E1" s="5" t="inlineStr">
         <is>
           <t>New/Renewal</t>
         </is>
       </c>
-      <c r="E1" s="5" t="inlineStr">
-        <is>
-          <t>Service / Package</t>
-        </is>
-      </c>
       <c r="F1" s="5" t="inlineStr">
         <is>
+          <t>Product</t>
+        </is>
+      </c>
+      <c r="G1" s="5" t="inlineStr">
+        <is>
           <t>Qty</t>
         </is>
       </c>
-      <c r="G1" s="5" t="inlineStr">
+      <c r="H1" s="5" t="inlineStr">
         <is>
           <t>Amount</t>
         </is>
       </c>
-      <c r="H1" s="5" t="inlineStr">
+      <c r="I1" s="5" t="inlineStr">
         <is>
           <t>Reference</t>
         </is>
       </c>
-      <c r="I1" s="5" t="inlineStr">
+      <c r="J1" s="5" t="inlineStr">
         <is>
           <t>Shared Reference</t>
         </is>
       </c>
-      <c r="J1" s="5" t="inlineStr">
+      <c r="K1" s="5" t="inlineStr">
         <is>
           <t>Split</t>
         </is>
       </c>
-      <c r="K1" s="5" t="inlineStr">
+      <c r="L1" s="5" t="inlineStr">
         <is>
           <t>Incentive</t>
         </is>
       </c>
-      <c r="L1" s="5" t="inlineStr">
+      <c r="M1" s="5" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>

</xml_diff>

<commit_message>
Round 7: invoices, Marketing Hub, Team Desk, clinic picker, recipe PDF steps
- Patient sale invoices (PDF + WhatsApp) with numbering, payment method and optional GST
- Marketing login role; Marketing Hub with lead sources, campaigns (cost per lead, ROI),
  content ideas with trending ideas, 7-day posting plan and hashtag sets
- Team Desk: tasks, attendance that fills paid days, monthly and per-member targets
- OPD clinic picker chips; clinic choice shown in every clinic booking
- What you sell lists product names with add buttons; Settings card to choose what
  shows on each dashboard (manager can customize too)
- Dashboard and team report KPIs follow the clinic's own product types
- Diet: step-by-step recipe PDFs, faster lists, contrast and overflow fixes
- Sheets: Campaigns, Tasks, Attendance (23 data sheets); APK 1.5

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014wSgWM4oMAShJr56qpgZfC
</commit_message>
<xml_diff>
--- a/admin/ThePrimeFit_Sheets.xlsx
+++ b/admin/ThePrimeFit_Sheets.xlsx
@@ -27,7 +27,10 @@
     <sheet name="Doctors" sheetId="18" state="visible" r:id="rId18"/>
     <sheet name="Content" sheetId="19" state="visible" r:id="rId19"/>
     <sheet name="Editors" sheetId="20" state="visible" r:id="rId20"/>
-    <sheet name="Activity Log" sheetId="21" state="visible" r:id="rId21"/>
+    <sheet name="Campaigns" sheetId="21" state="visible" r:id="rId21"/>
+    <sheet name="Tasks" sheetId="22" state="visible" r:id="rId22"/>
+    <sheet name="Attendance" sheetId="23" state="visible" r:id="rId23"/>
+    <sheet name="Activity Log" sheetId="24" state="visible" r:id="rId24"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -581,7 +584,7 @@
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>The app saves all data here. Each save rewrites the 20 sheets (Dashboard … Activity Log, including Service Sales, Other Sales, Doctors, Editors and Content), so edit data in the app, not in the sheets.</t>
+          <t>The app saves all data here. Each save rewrites the 23 sheets (Dashboard … Activity Log, including Service Sales, Other Sales, Doctors, Editors and Content), so edit data in the app, not in the sheets.</t>
         </is>
       </c>
     </row>
@@ -1928,7 +1931,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>2026-10-01T18:34:37.012Z</t>
+          <t>2026-10-01T19:17:21.198Z</t>
         </is>
       </c>
       <c r="C34" t="inlineStr"/>
@@ -1999,6 +2002,204 @@
 </file>
 
 <file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:M1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="15" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="10" max="10"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="12" customWidth="1" min="13" max="13"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="5" t="inlineStr">
+        <is>
+          <t>Campaign</t>
+        </is>
+      </c>
+      <c r="B1" s="5" t="inlineStr">
+        <is>
+          <t>Platform</t>
+        </is>
+      </c>
+      <c r="C1" s="5" t="inlineStr">
+        <is>
+          <t>Start</t>
+        </is>
+      </c>
+      <c r="D1" s="5" t="inlineStr">
+        <is>
+          <t>End</t>
+        </is>
+      </c>
+      <c r="E1" s="5" t="inlineStr">
+        <is>
+          <t>Budget</t>
+        </is>
+      </c>
+      <c r="F1" s="5" t="inlineStr">
+        <is>
+          <t>Spent</t>
+        </is>
+      </c>
+      <c r="G1" s="5" t="inlineStr">
+        <is>
+          <t>Leads</t>
+        </is>
+      </c>
+      <c r="H1" s="5" t="inlineStr">
+        <is>
+          <t>Converted</t>
+        </is>
+      </c>
+      <c r="I1" s="5" t="inlineStr">
+        <is>
+          <t>Cost per Lead</t>
+        </is>
+      </c>
+      <c r="J1" s="5" t="inlineStr">
+        <is>
+          <t>Revenue</t>
+        </is>
+      </c>
+      <c r="K1" s="5" t="inlineStr">
+        <is>
+          <t>ROI %</t>
+        </is>
+      </c>
+      <c r="L1" s="5" t="inlineStr">
+        <is>
+          <t>Goal</t>
+        </is>
+      </c>
+      <c r="M1" s="5" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="13" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="5" t="inlineStr">
+        <is>
+          <t>Task</t>
+        </is>
+      </c>
+      <c r="B1" s="5" t="inlineStr">
+        <is>
+          <t>Assigned To</t>
+        </is>
+      </c>
+      <c r="C1" s="5" t="inlineStr">
+        <is>
+          <t>Due</t>
+        </is>
+      </c>
+      <c r="D1" s="5" t="inlineStr">
+        <is>
+          <t>Priority</t>
+        </is>
+      </c>
+      <c r="E1" s="5" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="F1" s="5" t="inlineStr">
+        <is>
+          <t>Created By</t>
+        </is>
+      </c>
+      <c r="G1" s="5" t="inlineStr">
+        <is>
+          <t>Done By</t>
+        </is>
+      </c>
+      <c r="H1" s="5" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="13" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="5" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="B1" s="5" t="inlineStr">
+        <is>
+          <t>Team Member</t>
+        </is>
+      </c>
+      <c r="C1" s="5" t="inlineStr">
+        <is>
+          <t>Mark</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>

<commit_message>
Round 9: multiple founders, timed discussions, easier CRM, scroll fix
- Several founder profiles with profit share, monthly limits and capital in/out
- Founder Hub discussions saved with date, time and mode, attendees,
  outcome and next step; quick note box, search and a PDF of all discussions
- More Founder Hub content: month vs last month, money by mode, top lists
- Leads: quick add bar, one-tap call outcome after Call, next-stage button
- Fix page scrolling (overflow-x clip instead of hidden) on every screen
- Luxury styling for the new pieces; Founders sheet (26 sheets); APK 1.7

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014wSgWM4oMAShJr56qpgZfC
</commit_message>
<xml_diff>
--- a/admin/ThePrimeFit_Sheets.xlsx
+++ b/admin/ThePrimeFit_Sheets.xlsx
@@ -31,8 +31,9 @@
     <sheet name="Ads Report" sheetId="22" state="visible" r:id="rId22"/>
     <sheet name="Tasks" sheetId="23" state="visible" r:id="rId23"/>
     <sheet name="Attendance" sheetId="24" state="visible" r:id="rId24"/>
-    <sheet name="Founder Notes" sheetId="25" state="visible" r:id="rId25"/>
-    <sheet name="Activity Log" sheetId="26" state="visible" r:id="rId26"/>
+    <sheet name="Founders" sheetId="25" state="visible" r:id="rId25"/>
+    <sheet name="Founder Notes" sheetId="26" state="visible" r:id="rId26"/>
+    <sheet name="Activity Log" sheetId="27" state="visible" r:id="rId27"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -586,7 +587,7 @@
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>The app saves all data here. Each save rewrites the 25 sheets (Dashboard … Activity Log, including Service Sales, Other Sales, Doctors, Editors and Content), so edit data in the app, not in the sheets.</t>
+          <t>The app saves all data here. Each save rewrites the 26 sheets (Dashboard … Activity Log, including Service Sales, Other Sales, Doctors, Editors and Content), so edit data in the app, not in the sheets.</t>
         </is>
       </c>
     </row>
@@ -1236,7 +1237,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I1"/>
+  <dimension ref="A1:J1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1244,10 +1245,11 @@
     <col width="12" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="16" customWidth="1" min="6" max="6"/>
-    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
     <col width="12" customWidth="1" min="8" max="8"/>
-    <col width="19" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="19" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1263,35 +1265,40 @@
       </c>
       <c r="C1" s="5" t="inlineStr">
         <is>
+          <t>Founder</t>
+        </is>
+      </c>
+      <c r="D1" s="5" t="inlineStr">
+        <is>
           <t>Category</t>
         </is>
       </c>
-      <c r="D1" s="5" t="inlineStr">
+      <c r="E1" s="5" t="inlineStr">
         <is>
           <t>Name</t>
         </is>
       </c>
-      <c r="E1" s="5" t="inlineStr">
+      <c r="F1" s="5" t="inlineStr">
         <is>
           <t>Amount</t>
         </is>
       </c>
-      <c r="F1" s="5" t="inlineStr">
+      <c r="G1" s="5" t="inlineStr">
         <is>
           <t>Payment Method</t>
         </is>
       </c>
-      <c r="G1" s="5" t="inlineStr">
+      <c r="H1" s="5" t="inlineStr">
         <is>
           <t>Note</t>
         </is>
       </c>
-      <c r="H1" s="5" t="inlineStr">
+      <c r="I1" s="5" t="inlineStr">
         <is>
           <t>Counted</t>
         </is>
       </c>
-      <c r="I1" s="5" t="inlineStr">
+      <c r="J1" s="5" t="inlineStr">
         <is>
           <t>Ad Leads (manual)</t>
         </is>
@@ -1945,7 +1952,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>2026-10-01T20:05:54.070Z</t>
+          <t>2026-10-01T20:37:27.726Z</t>
         </is>
       </c>
       <c r="C34" t="inlineStr"/>
@@ -2285,7 +2292,118 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1"/>
+  <dimension ref="A1:K3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="17" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="13" customWidth="1" min="10" max="10"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="5" t="inlineStr">
+        <is>
+          <t>Founder</t>
+        </is>
+      </c>
+      <c r="B1" s="5" t="inlineStr">
+        <is>
+          <t>Title</t>
+        </is>
+      </c>
+      <c r="C1" s="5" t="inlineStr">
+        <is>
+          <t>Mobile</t>
+        </is>
+      </c>
+      <c r="D1" s="5" t="inlineStr">
+        <is>
+          <t>Profit Share %</t>
+        </is>
+      </c>
+      <c r="E1" s="5" t="inlineStr">
+        <is>
+          <t>Monthly Limit</t>
+        </is>
+      </c>
+      <c r="F1" s="5" t="inlineStr">
+        <is>
+          <t>Spent (all time)</t>
+        </is>
+      </c>
+      <c r="G1" s="5" t="inlineStr">
+        <is>
+          <t>Spent this month</t>
+        </is>
+      </c>
+      <c r="H1" s="5" t="inlineStr">
+        <is>
+          <t>Invested</t>
+        </is>
+      </c>
+      <c r="I1" s="5" t="inlineStr">
+        <is>
+          <t>Withdrawn</t>
+        </is>
+      </c>
+      <c r="J1" s="5" t="inlineStr">
+        <is>
+          <t>Net Capital</t>
+        </is>
+      </c>
+      <c r="K1" s="5" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Capital entries</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Amount</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:N1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2296,6 +2414,12 @@
     <col width="12" customWidth="1" min="6" max="6"/>
     <col width="12" customWidth="1" min="7" max="7"/>
     <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="20" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="10" max="10"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="12" customWidth="1" min="13" max="13"/>
+    <col width="12" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2306,35 +2430,65 @@
       </c>
       <c r="B1" s="5" t="inlineStr">
         <is>
+          <t>Time</t>
+        </is>
+      </c>
+      <c r="C1" s="5" t="inlineStr">
+        <is>
+          <t>Mode</t>
+        </is>
+      </c>
+      <c r="D1" s="5" t="inlineStr">
+        <is>
           <t>Type</t>
         </is>
       </c>
-      <c r="C1" s="5" t="inlineStr">
+      <c r="E1" s="5" t="inlineStr">
         <is>
           <t>Title</t>
         </is>
       </c>
-      <c r="D1" s="5" t="inlineStr">
-        <is>
-          <t>Note</t>
-        </is>
-      </c>
-      <c r="E1" s="5" t="inlineStr">
+      <c r="F1" s="5" t="inlineStr">
+        <is>
+          <t>Details</t>
+        </is>
+      </c>
+      <c r="G1" s="5" t="inlineStr">
+        <is>
+          <t>With</t>
+        </is>
+      </c>
+      <c r="H1" s="5" t="inlineStr">
+        <is>
+          <t>Minutes</t>
+        </is>
+      </c>
+      <c r="I1" s="5" t="inlineStr">
+        <is>
+          <t>Outcome / Decision</t>
+        </is>
+      </c>
+      <c r="J1" s="5" t="inlineStr">
+        <is>
+          <t>Next Step</t>
+        </is>
+      </c>
+      <c r="K1" s="5" t="inlineStr">
         <is>
           <t>Due</t>
         </is>
       </c>
-      <c r="F1" s="5" t="inlineStr">
+      <c r="L1" s="5" t="inlineStr">
         <is>
           <t>Pinned</t>
         </is>
       </c>
-      <c r="G1" s="5" t="inlineStr">
+      <c r="M1" s="5" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="H1" s="5" t="inlineStr">
+      <c r="N1" s="5" t="inlineStr">
         <is>
           <t>By</t>
         </is>
@@ -2345,7 +2499,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet27.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>

<commit_message>
Serial slip numbers, Slips sheet, no-signature digital slips; APK 2.2
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014wSgWM4oMAShJr56qpgZfC
</commit_message>
<xml_diff>
--- a/admin/ThePrimeFit_Sheets.xlsx
+++ b/admin/ThePrimeFit_Sheets.xlsx
@@ -33,7 +33,8 @@
     <sheet name="Attendance" sheetId="24" state="visible" r:id="rId24"/>
     <sheet name="Founders" sheetId="25" state="visible" r:id="rId25"/>
     <sheet name="Founder Notes" sheetId="26" state="visible" r:id="rId26"/>
-    <sheet name="Activity Log" sheetId="27" state="visible" r:id="rId27"/>
+    <sheet name="Slips" sheetId="27" state="visible" r:id="rId27"/>
+    <sheet name="Activity Log" sheetId="28" state="visible" r:id="rId28"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -587,7 +588,7 @@
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>The app saves all data here. Each save rewrites the 26 sheets (Dashboard … Activity Log, including Service Sales, Other Sales, Doctors, Editors and Content), so edit data in the app, not in the sheets.</t>
+          <t>The app saves all data here. Each save rewrites the 27 sheets (Dashboard … Activity Log, including Service Sales, Other Sales, Doctors, Editors, Content and Slips), so edit data in the app, not in the sheets.</t>
         </is>
       </c>
     </row>
@@ -897,13 +898,11 @@
           <t>Unlimited</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr"/>
       <c r="J2" t="inlineStr">
         <is>
           <t>Service</t>
         </is>
       </c>
-      <c r="K2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -938,13 +937,11 @@
           <t>Unlimited</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr"/>
       <c r="J3" t="inlineStr">
         <is>
           <t>Service</t>
         </is>
       </c>
-      <c r="K3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -979,13 +976,11 @@
           <t>Unlimited</t>
         </is>
       </c>
-      <c r="I4" t="inlineStr"/>
       <c r="J4" t="inlineStr">
         <is>
           <t>Service</t>
         </is>
       </c>
-      <c r="K4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1020,13 +1015,11 @@
           <t>Unlimited</t>
         </is>
       </c>
-      <c r="I5" t="inlineStr"/>
       <c r="J5" t="inlineStr">
         <is>
           <t>Service</t>
         </is>
       </c>
-      <c r="K5" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1738,8 +1731,6 @@
           <t>Order Required</t>
         </is>
       </c>
-      <c r="B16" t="inlineStr"/>
-      <c r="C16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1838,8 +1829,6 @@
           <t>Top Performer</t>
         </is>
       </c>
-      <c r="B24" t="inlineStr"/>
-      <c r="C24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -1850,7 +1839,6 @@
       <c r="B25" t="n">
         <v>0</v>
       </c>
-      <c r="C25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -1861,7 +1849,6 @@
       <c r="B26" t="n">
         <v>0</v>
       </c>
-      <c r="C26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -1872,7 +1859,6 @@
       <c r="B27" t="n">
         <v>0</v>
       </c>
-      <c r="C27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -1883,7 +1869,6 @@
       <c r="B28" t="n">
         <v>0</v>
       </c>
-      <c r="C28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -1894,7 +1879,6 @@
       <c r="B29" t="n">
         <v>0</v>
       </c>
-      <c r="C29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -1902,8 +1886,6 @@
           <t>Low Stock Alerts</t>
         </is>
       </c>
-      <c r="B30" t="inlineStr"/>
-      <c r="C30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -1955,7 +1937,6 @@
           <t>2026-10-01T20:37:27.726Z</t>
         </is>
       </c>
-      <c r="C34" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2500,6 +2481,90 @@
 </file>
 
 <file path=xl/worksheets/sheet27.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:K1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="40" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="10" max="10"/>
+    <col width="21" customWidth="1" min="11" max="11"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="5" t="inlineStr">
+        <is>
+          <t>Slip No.</t>
+        </is>
+      </c>
+      <c r="B1" s="5" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="C1" s="5" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="D1" s="5" t="inlineStr">
+        <is>
+          <t>Patient</t>
+        </is>
+      </c>
+      <c r="E1" s="5" t="inlineStr">
+        <is>
+          <t>Mobile</t>
+        </is>
+      </c>
+      <c r="F1" s="5" t="inlineStr">
+        <is>
+          <t>Items</t>
+        </is>
+      </c>
+      <c r="G1" s="5" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="H1" s="5" t="inlineStr">
+        <is>
+          <t>Payment</t>
+        </is>
+      </c>
+      <c r="I1" s="5" t="inlineStr">
+        <is>
+          <t>Made By</t>
+        </is>
+      </c>
+      <c r="J1" s="5" t="inlineStr">
+        <is>
+          <t>Made On</t>
+        </is>
+      </c>
+      <c r="K1" s="5" t="inlineStr">
+        <is>
+          <t>Sale Invoice Nos.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet28.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>